<commit_message>
created common template blocks
</commit_message>
<xml_diff>
--- a/taekook_universe.xlsx
+++ b/taekook_universe.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/haripriyakrishnan/Downloads/Python/taekook_universe/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0358ADC-379E-5843-8029-DBEFEACB9C2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA3045E0-09B7-A847-B00D-B9A27A83A502}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="15020" yWindow="3080" windowWidth="22560" windowHeight="17440" activeTab="7" xr2:uid="{52A6CF0C-9FDF-6A4B-B1CC-CBEE960F6C98}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="933" uniqueCount="612">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="934" uniqueCount="612">
   <si>
     <t>Jungkook</t>
   </si>
@@ -20596,6 +20596,9 @@
       <c r="D4" t="s">
         <v>476</v>
       </c>
+      <c r="E4" t="s">
+        <v>476</v>
+      </c>
       <c r="F4" t="s">
         <v>487</v>
       </c>

</xml_diff>